<commit_message>
Fix Kohler product mapping, pricing, and image path handling
</commit_message>
<xml_diff>
--- a/backend/kohler_catalog_full.xlsx
+++ b/backend/kohler_catalog_full.xlsx
@@ -4377,7 +4377,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>16346</v>
+        <v>4300</v>
       </c>
       <c r="I88" t="inlineStr">
         <is>
@@ -4516,7 +4516,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>16347</v>
+        <v>4300</v>
       </c>
       <c r="I91" t="inlineStr">
         <is>
@@ -14270,7 +14270,7 @@
         </is>
       </c>
       <c r="H299" t="n">
-        <v>24431</v>
+        <v>14700</v>
       </c>
       <c r="I299" t="inlineStr">
         <is>
@@ -14313,7 +14313,7 @@
         </is>
       </c>
       <c r="H300" t="n">
-        <v>24431</v>
+        <v>16300</v>
       </c>
       <c r="I300" t="inlineStr">
         <is>
@@ -14356,7 +14356,7 @@
         </is>
       </c>
       <c r="H301" t="n">
-        <v>24431</v>
+        <v>17500</v>
       </c>
       <c r="I301" t="inlineStr">
         <is>
@@ -14399,7 +14399,7 @@
         </is>
       </c>
       <c r="H302" t="n">
-        <v>24431</v>
+        <v>17500</v>
       </c>
       <c r="I302" t="inlineStr">
         <is>
@@ -14442,7 +14442,7 @@
         </is>
       </c>
       <c r="H303" t="n">
-        <v>24431</v>
+        <v>11700</v>
       </c>
       <c r="I303" t="inlineStr">
         <is>
@@ -14485,7 +14485,7 @@
         </is>
       </c>
       <c r="H304" t="n">
-        <v>24431</v>
+        <v>16300</v>
       </c>
       <c r="I304" t="inlineStr">
         <is>
@@ -52884,7 +52884,7 @@
         </is>
       </c>
       <c r="H1147" t="n">
-        <v>54000</v>
+        <v>106100</v>
       </c>
       <c r="I1147" t="inlineStr">
         <is>
@@ -56787,7 +56787,7 @@
         </is>
       </c>
       <c r="H1233" t="n">
-        <v>47080</v>
+        <v>55000</v>
       </c>
       <c r="I1233" t="inlineStr">
         <is>
@@ -56979,7 +56979,7 @@
         </is>
       </c>
       <c r="H1237" t="n">
-        <v>47080</v>
+        <v>60500</v>
       </c>
       <c r="I1237" t="inlineStr">
         <is>
@@ -57027,7 +57027,7 @@
         </is>
       </c>
       <c r="H1238" t="n">
-        <v>47080</v>
+        <v>60500</v>
       </c>
       <c r="I1238" t="inlineStr">
         <is>
@@ -57075,7 +57075,7 @@
         </is>
       </c>
       <c r="H1239" t="n">
-        <v>47080</v>
+        <v>60500</v>
       </c>
       <c r="I1239" t="inlineStr">
         <is>
@@ -57530,7 +57530,7 @@
         </is>
       </c>
       <c r="H1249" t="n">
-        <v>55000</v>
+        <v>60500</v>
       </c>
       <c r="I1249" t="inlineStr">
         <is>
@@ -57626,7 +57626,7 @@
         </is>
       </c>
       <c r="H1251" t="n">
-        <v>55000</v>
+        <v>60500</v>
       </c>
       <c r="I1251" t="inlineStr">
         <is>
@@ -57722,7 +57722,7 @@
         </is>
       </c>
       <c r="H1253" t="n">
-        <v>55000</v>
+        <v>60500</v>
       </c>
       <c r="I1253" t="inlineStr">
         <is>

</xml_diff>